<commit_message>
update Excel templates for AM Report and Mud Resistivity
</commit_message>
<xml_diff>
--- a/priv/python/excel_templates/TEMPLATE_AM Report.xlsx
+++ b/priv/python/excel_templates/TEMPLATE_AM Report.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deanerfree/projects/elixir/suncor-project-spinup/priv/python/excel_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF9579C-9241-674B-B330-B5225A154630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DD3886-3DC1-914E-AB22-F9136E74FDC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3420" yWindow="660" windowWidth="19100" windowHeight="13900" xr2:uid="{26F572F5-B233-44A0-940B-1963B58B7EF0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Mar 04" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="71">
   <si>
     <t>DAILY GEOLOGICAL REPORT</t>
   </si>
@@ -246,7 +246,10 @@
     <t>Lower Wab/ RMZ Top</t>
   </si>
   <si>
-    <t>Production Casing</t>
+    <t>Intermediate Hole</t>
+  </si>
+  <si>
+    <t>Intermediate Casing</t>
   </si>
 </sst>
 </file>
@@ -1082,6 +1085,268 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1177,13 +1442,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1209,264 +1467,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1920,223 +1923,223 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22" x14ac:dyDescent="0.3">
-      <c r="A1" s="26"/>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="30" t="s">
+      <c r="A1" s="104"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="32"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+      <c r="G1" s="109"/>
+      <c r="H1" s="109"/>
+      <c r="I1" s="109"/>
+      <c r="J1" s="109"/>
+      <c r="K1" s="110"/>
       <c r="L1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="33"/>
-      <c r="N1" s="34"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="112"/>
     </row>
     <row r="2" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="38" t="s">
+      <c r="A2" s="106"/>
+      <c r="B2" s="107"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="114"/>
+      <c r="F2" s="114"/>
+      <c r="G2" s="114"/>
+      <c r="H2" s="114"/>
+      <c r="I2" s="114"/>
+      <c r="J2" s="114"/>
+      <c r="K2" s="115"/>
+      <c r="L2" s="116" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="39"/>
+      <c r="M2" s="117"/>
       <c r="N2" s="15"/>
     </row>
     <row r="3" spans="1:14" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="43" t="s">
+      <c r="A3" s="106"/>
+      <c r="B3" s="107"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="118"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
+      <c r="H3" s="119"/>
+      <c r="I3" s="119"/>
+      <c r="J3" s="119"/>
+      <c r="K3" s="120"/>
+      <c r="L3" s="121" t="s">
         <v>56</v>
       </c>
-      <c r="M3" s="44"/>
+      <c r="M3" s="122"/>
       <c r="N3" s="16"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="60"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60" t="s">
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="136"/>
+      <c r="F4" s="136"/>
+      <c r="G4" s="136"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
+      <c r="K4" s="136"/>
+      <c r="L4" s="136" t="s">
         <v>62</v>
       </c>
-      <c r="M4" s="60"/>
-      <c r="N4" s="61"/>
+      <c r="M4" s="136"/>
+      <c r="N4" s="137"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="64" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="65" t="s">
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="66"/>
-      <c r="J5" s="66"/>
-      <c r="K5" s="66"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="58"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="138"/>
+      <c r="J5" s="138"/>
+      <c r="K5" s="138"/>
+      <c r="L5" s="89"/>
+      <c r="M5" s="89"/>
+      <c r="N5" s="134"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="123" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="47" t="s">
+      <c r="B6" s="124"/>
+      <c r="C6" s="125" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="48"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="53" t="s">
+      <c r="D6" s="126"/>
+      <c r="E6" s="127"/>
+      <c r="F6" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="53"/>
+      <c r="G6" s="98"/>
       <c r="H6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="55"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="57"/>
+      <c r="I6" s="89"/>
+      <c r="J6" s="89"/>
+      <c r="K6" s="89"/>
+      <c r="L6" s="131"/>
+      <c r="M6" s="132"/>
+      <c r="N6" s="133"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" s="45"/>
-      <c r="B7" s="46"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
+      <c r="A7" s="123"/>
+      <c r="B7" s="124"/>
+      <c r="C7" s="128"/>
+      <c r="D7" s="129"/>
+      <c r="E7" s="130"/>
+      <c r="F7" s="98"/>
+      <c r="G7" s="98"/>
       <c r="H7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="54"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="54"/>
-      <c r="L7" s="54"/>
-      <c r="M7" s="54"/>
-      <c r="N7" s="58"/>
+      <c r="I7" s="89"/>
+      <c r="J7" s="89"/>
+      <c r="K7" s="89"/>
+      <c r="L7" s="89"/>
+      <c r="M7" s="89"/>
+      <c r="N7" s="134"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" s="73" t="s">
+      <c r="A8" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="53"/>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-      <c r="F8" s="53" t="s">
+      <c r="B8" s="98"/>
+      <c r="C8" s="99"/>
+      <c r="D8" s="99"/>
+      <c r="E8" s="99"/>
+      <c r="F8" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="53"/>
+      <c r="G8" s="98"/>
       <c r="H8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="54"/>
-      <c r="J8" s="54"/>
-      <c r="K8" s="54"/>
-      <c r="L8" s="75" t="s">
+      <c r="I8" s="89"/>
+      <c r="J8" s="89"/>
+      <c r="K8" s="89"/>
+      <c r="L8" s="100" t="s">
         <v>55</v>
       </c>
-      <c r="M8" s="76"/>
-      <c r="N8" s="77"/>
+      <c r="M8" s="101"/>
+      <c r="N8" s="102"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" s="73"/>
-      <c r="B9" s="53"/>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="53"/>
-      <c r="G9" s="53"/>
+      <c r="A9" s="97"/>
+      <c r="B9" s="98"/>
+      <c r="C9" s="99"/>
+      <c r="D9" s="99"/>
+      <c r="E9" s="99"/>
+      <c r="F9" s="98"/>
+      <c r="G9" s="98"/>
       <c r="H9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="54"/>
-      <c r="J9" s="54"/>
-      <c r="K9" s="54"/>
-      <c r="L9" s="74"/>
-      <c r="M9" s="74"/>
-      <c r="N9" s="78"/>
+      <c r="I9" s="89"/>
+      <c r="J9" s="89"/>
+      <c r="K9" s="89"/>
+      <c r="L9" s="99"/>
+      <c r="M9" s="99"/>
+      <c r="N9" s="103"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10" s="67" t="s">
+      <c r="A10" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="68"/>
-      <c r="G10" s="68"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="68"/>
-      <c r="J10" s="68"/>
-      <c r="K10" s="68"/>
-      <c r="L10" s="68"/>
-      <c r="M10" s="68"/>
-      <c r="N10" s="69"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="28"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" s="62" t="s">
+      <c r="A11" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="63" t="s">
+      <c r="B11" s="87"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="89"/>
+      <c r="E11" s="87" t="s">
         <v>63</v>
       </c>
-      <c r="F11" s="63"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="71"/>
-      <c r="I11" s="71"/>
-      <c r="J11" s="65" t="s">
+      <c r="F11" s="87"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="K11" s="72"/>
+      <c r="K11" s="96"/>
       <c r="L11" s="3" t="s">
         <v>28</v>
       </c>
@@ -2148,402 +2151,404 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A12" s="62" t="s">
+      <c r="A12" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="63" t="s">
+      <c r="B12" s="87"/>
+      <c r="C12" s="89"/>
+      <c r="D12" s="89"/>
+      <c r="E12" s="87" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="63"/>
-      <c r="G12" s="71"/>
-      <c r="H12" s="71"/>
-      <c r="I12" s="71"/>
-      <c r="J12" s="63" t="s">
+      <c r="F12" s="87"/>
+      <c r="G12" s="88"/>
+      <c r="H12" s="88"/>
+      <c r="I12" s="88"/>
+      <c r="J12" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="K12" s="63"/>
+      <c r="K12" s="87"/>
       <c r="L12" s="14"/>
       <c r="M12" s="14"/>
       <c r="N12" s="9"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A13" s="62" t="s">
+      <c r="A13" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79"/>
-      <c r="E13" s="63" t="s">
+      <c r="B13" s="87"/>
+      <c r="C13" s="94"/>
+      <c r="D13" s="94"/>
+      <c r="E13" s="87" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="63"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="63" t="s">
+      <c r="F13" s="87"/>
+      <c r="G13" s="89"/>
+      <c r="H13" s="89"/>
+      <c r="I13" s="89"/>
+      <c r="J13" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="K13" s="63"/>
+      <c r="K13" s="87"/>
       <c r="L13" s="14"/>
       <c r="M13" s="14"/>
       <c r="N13" s="9"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A14" s="62" t="s">
+      <c r="A14" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="71"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="63" t="s">
+      <c r="B14" s="87"/>
+      <c r="C14" s="88"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="63"/>
-      <c r="G14" s="83"/>
-      <c r="H14" s="83"/>
-      <c r="I14" s="83"/>
-      <c r="J14" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="K14" s="63"/>
+      <c r="F14" s="87"/>
+      <c r="G14" s="93"/>
+      <c r="H14" s="93"/>
+      <c r="I14" s="93"/>
+      <c r="J14" s="87" t="s">
+        <v>69</v>
+      </c>
+      <c r="K14" s="87"/>
       <c r="L14" s="14"/>
       <c r="M14" s="14"/>
       <c r="N14" s="9"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="71"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="63" t="s">
+      <c r="B15" s="87"/>
+      <c r="C15" s="88"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="63"/>
-      <c r="G15" s="54" t="s">
+      <c r="F15" s="87"/>
+      <c r="G15" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="63" t="s">
-        <v>69</v>
-      </c>
-      <c r="K15" s="63"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="87" t="s">
+        <v>70</v>
+      </c>
+      <c r="K15" s="87"/>
       <c r="L15" s="14"/>
       <c r="M15" s="14"/>
       <c r="N15" s="9"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A16" s="62" t="s">
+      <c r="A16" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="71" t="str">
+      <c r="B16" s="87"/>
+      <c r="C16" s="88" t="str">
         <f>IF(C$15="","",C$14-C$15)</f>
         <v/>
       </c>
-      <c r="D16" s="71"/>
-      <c r="E16" s="63" t="s">
+      <c r="D16" s="88"/>
+      <c r="E16" s="87" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="63"/>
-      <c r="G16" s="54" t="s">
+      <c r="F16" s="87"/>
+      <c r="G16" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="H16" s="54"/>
-      <c r="I16" s="54"/>
-      <c r="J16" s="63"/>
-      <c r="K16" s="63"/>
+      <c r="H16" s="89"/>
+      <c r="I16" s="89"/>
+      <c r="J16" s="87" t="s">
+        <v>26</v>
+      </c>
+      <c r="K16" s="87"/>
       <c r="L16" s="14"/>
       <c r="M16" s="14"/>
       <c r="N16" s="9"/>
     </row>
     <row r="17" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="80" t="s">
+      <c r="A17" s="90" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="81"/>
-      <c r="C17" s="81"/>
-      <c r="D17" s="81"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="81"/>
-      <c r="G17" s="81"/>
-      <c r="H17" s="81"/>
-      <c r="I17" s="81"/>
-      <c r="J17" s="81"/>
-      <c r="K17" s="81"/>
-      <c r="L17" s="81"/>
-      <c r="M17" s="81"/>
-      <c r="N17" s="82"/>
+      <c r="B17" s="91"/>
+      <c r="C17" s="91"/>
+      <c r="D17" s="91"/>
+      <c r="E17" s="91"/>
+      <c r="F17" s="91"/>
+      <c r="G17" s="91"/>
+      <c r="H17" s="91"/>
+      <c r="I17" s="91"/>
+      <c r="J17" s="91"/>
+      <c r="K17" s="91"/>
+      <c r="L17" s="91"/>
+      <c r="M17" s="91"/>
+      <c r="N17" s="92"/>
     </row>
     <row r="18" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="92"/>
-      <c r="B18" s="93"/>
-      <c r="C18" s="93"/>
-      <c r="D18" s="93"/>
-      <c r="E18" s="93"/>
-      <c r="F18" s="93"/>
-      <c r="G18" s="93"/>
-      <c r="H18" s="93"/>
-      <c r="I18" s="93"/>
-      <c r="J18" s="93"/>
-      <c r="K18" s="93"/>
-      <c r="L18" s="93"/>
-      <c r="M18" s="93"/>
-      <c r="N18" s="94"/>
+      <c r="A18" s="71"/>
+      <c r="B18" s="72"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="72"/>
+      <c r="F18" s="72"/>
+      <c r="G18" s="72"/>
+      <c r="H18" s="72"/>
+      <c r="I18" s="72"/>
+      <c r="J18" s="72"/>
+      <c r="K18" s="72"/>
+      <c r="L18" s="72"/>
+      <c r="M18" s="72"/>
+      <c r="N18" s="73"/>
     </row>
     <row r="19" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="95" t="s">
+      <c r="A19" s="74" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="96"/>
-      <c r="C19" s="96"/>
-      <c r="D19" s="96"/>
-      <c r="E19" s="96"/>
-      <c r="F19" s="96"/>
-      <c r="G19" s="96"/>
-      <c r="H19" s="96"/>
-      <c r="I19" s="96"/>
-      <c r="J19" s="96"/>
-      <c r="K19" s="96"/>
-      <c r="L19" s="96"/>
-      <c r="M19" s="96"/>
-      <c r="N19" s="97"/>
+      <c r="B19" s="75"/>
+      <c r="C19" s="75"/>
+      <c r="D19" s="75"/>
+      <c r="E19" s="75"/>
+      <c r="F19" s="75"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="75"/>
+      <c r="I19" s="75"/>
+      <c r="J19" s="75"/>
+      <c r="K19" s="75"/>
+      <c r="L19" s="75"/>
+      <c r="M19" s="75"/>
+      <c r="N19" s="76"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A20" s="98"/>
-      <c r="B20" s="99"/>
-      <c r="C20" s="99"/>
-      <c r="D20" s="99"/>
-      <c r="E20" s="99"/>
-      <c r="F20" s="99"/>
-      <c r="G20" s="99"/>
-      <c r="H20" s="99"/>
-      <c r="I20" s="99"/>
-      <c r="J20" s="99"/>
-      <c r="K20" s="99"/>
-      <c r="L20" s="99"/>
-      <c r="M20" s="99"/>
-      <c r="N20" s="100"/>
+      <c r="A20" s="77"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="78"/>
+      <c r="E20" s="78"/>
+      <c r="F20" s="78"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="78"/>
+      <c r="I20" s="78"/>
+      <c r="J20" s="78"/>
+      <c r="K20" s="78"/>
+      <c r="L20" s="78"/>
+      <c r="M20" s="78"/>
+      <c r="N20" s="79"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A21" s="101"/>
-      <c r="B21" s="102"/>
-      <c r="C21" s="102"/>
-      <c r="D21" s="102"/>
-      <c r="E21" s="102"/>
-      <c r="F21" s="102"/>
-      <c r="G21" s="102"/>
-      <c r="H21" s="102"/>
-      <c r="I21" s="102"/>
-      <c r="J21" s="102"/>
-      <c r="K21" s="102"/>
-      <c r="L21" s="102"/>
-      <c r="M21" s="102"/>
-      <c r="N21" s="103"/>
+      <c r="A21" s="80"/>
+      <c r="B21" s="81"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="81"/>
+      <c r="E21" s="81"/>
+      <c r="F21" s="81"/>
+      <c r="G21" s="81"/>
+      <c r="H21" s="81"/>
+      <c r="I21" s="81"/>
+      <c r="J21" s="81"/>
+      <c r="K21" s="81"/>
+      <c r="L21" s="81"/>
+      <c r="M21" s="81"/>
+      <c r="N21" s="82"/>
     </row>
     <row r="22" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="101"/>
-      <c r="B22" s="102"/>
-      <c r="C22" s="102"/>
-      <c r="D22" s="102"/>
-      <c r="E22" s="102"/>
-      <c r="F22" s="102"/>
-      <c r="G22" s="102"/>
-      <c r="H22" s="102"/>
-      <c r="I22" s="102"/>
-      <c r="J22" s="102"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="102"/>
-      <c r="M22" s="102"/>
-      <c r="N22" s="103"/>
+      <c r="A22" s="80"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
+      <c r="E22" s="81"/>
+      <c r="F22" s="81"/>
+      <c r="G22" s="81"/>
+      <c r="H22" s="81"/>
+      <c r="I22" s="81"/>
+      <c r="J22" s="81"/>
+      <c r="K22" s="81"/>
+      <c r="L22" s="81"/>
+      <c r="M22" s="81"/>
+      <c r="N22" s="82"/>
     </row>
     <row r="23" spans="1:14" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="101"/>
-      <c r="B23" s="102"/>
-      <c r="C23" s="102"/>
-      <c r="D23" s="102"/>
-      <c r="E23" s="102"/>
-      <c r="F23" s="102"/>
-      <c r="G23" s="102"/>
-      <c r="H23" s="102"/>
-      <c r="I23" s="102"/>
-      <c r="J23" s="102"/>
-      <c r="K23" s="102"/>
-      <c r="L23" s="102"/>
-      <c r="M23" s="102"/>
-      <c r="N23" s="103"/>
+      <c r="A23" s="80"/>
+      <c r="B23" s="81"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="81"/>
+      <c r="F23" s="81"/>
+      <c r="G23" s="81"/>
+      <c r="H23" s="81"/>
+      <c r="I23" s="81"/>
+      <c r="J23" s="81"/>
+      <c r="K23" s="81"/>
+      <c r="L23" s="81"/>
+      <c r="M23" s="81"/>
+      <c r="N23" s="82"/>
     </row>
     <row r="24" spans="1:14" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="104"/>
-      <c r="B24" s="105"/>
-      <c r="C24" s="105"/>
-      <c r="D24" s="105"/>
-      <c r="E24" s="105"/>
-      <c r="F24" s="105"/>
-      <c r="G24" s="105"/>
-      <c r="H24" s="105"/>
-      <c r="I24" s="105"/>
-      <c r="J24" s="105"/>
-      <c r="K24" s="105"/>
-      <c r="L24" s="105"/>
-      <c r="M24" s="105"/>
-      <c r="N24" s="106"/>
+      <c r="A24" s="83"/>
+      <c r="B24" s="84"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="84"/>
+      <c r="E24" s="84"/>
+      <c r="F24" s="84"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="84"/>
+      <c r="I24" s="84"/>
+      <c r="J24" s="84"/>
+      <c r="K24" s="84"/>
+      <c r="L24" s="84"/>
+      <c r="M24" s="84"/>
+      <c r="N24" s="85"/>
     </row>
     <row r="25" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="95" t="s">
+      <c r="A25" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="96"/>
-      <c r="C25" s="96"/>
-      <c r="D25" s="96"/>
-      <c r="E25" s="96"/>
-      <c r="F25" s="96"/>
-      <c r="G25" s="96"/>
-      <c r="H25" s="96"/>
-      <c r="I25" s="96"/>
-      <c r="J25" s="96"/>
-      <c r="K25" s="96"/>
-      <c r="L25" s="96"/>
-      <c r="M25" s="96"/>
-      <c r="N25" s="97"/>
+      <c r="B25" s="75"/>
+      <c r="C25" s="75"/>
+      <c r="D25" s="75"/>
+      <c r="E25" s="75"/>
+      <c r="F25" s="75"/>
+      <c r="G25" s="75"/>
+      <c r="H25" s="75"/>
+      <c r="I25" s="75"/>
+      <c r="J25" s="75"/>
+      <c r="K25" s="75"/>
+      <c r="L25" s="75"/>
+      <c r="M25" s="75"/>
+      <c r="N25" s="76"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A26" s="98"/>
-      <c r="B26" s="99"/>
-      <c r="C26" s="99"/>
-      <c r="D26" s="99"/>
-      <c r="E26" s="99"/>
-      <c r="F26" s="99"/>
-      <c r="G26" s="99"/>
-      <c r="H26" s="99"/>
-      <c r="I26" s="99"/>
-      <c r="J26" s="99"/>
-      <c r="K26" s="99"/>
-      <c r="L26" s="99"/>
-      <c r="M26" s="99"/>
-      <c r="N26" s="100"/>
+      <c r="A26" s="77"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="78"/>
+      <c r="J26" s="78"/>
+      <c r="K26" s="78"/>
+      <c r="L26" s="78"/>
+      <c r="M26" s="78"/>
+      <c r="N26" s="79"/>
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="101"/>
-      <c r="B27" s="102"/>
-      <c r="C27" s="102"/>
-      <c r="D27" s="102"/>
-      <c r="E27" s="102"/>
-      <c r="F27" s="102"/>
-      <c r="G27" s="102"/>
-      <c r="H27" s="102"/>
-      <c r="I27" s="102"/>
-      <c r="J27" s="102"/>
-      <c r="K27" s="102"/>
-      <c r="L27" s="102"/>
-      <c r="M27" s="102"/>
-      <c r="N27" s="103"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="81"/>
+      <c r="C27" s="81"/>
+      <c r="D27" s="81"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="81"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
+      <c r="I27" s="81"/>
+      <c r="J27" s="81"/>
+      <c r="K27" s="81"/>
+      <c r="L27" s="81"/>
+      <c r="M27" s="81"/>
+      <c r="N27" s="82"/>
     </row>
     <row r="28" spans="1:14" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="101"/>
-      <c r="B28" s="102"/>
-      <c r="C28" s="102"/>
-      <c r="D28" s="102"/>
-      <c r="E28" s="102"/>
-      <c r="F28" s="102"/>
-      <c r="G28" s="102"/>
-      <c r="H28" s="102"/>
-      <c r="I28" s="102"/>
-      <c r="J28" s="102"/>
-      <c r="K28" s="102"/>
-      <c r="L28" s="102"/>
-      <c r="M28" s="102"/>
-      <c r="N28" s="103"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="81"/>
+      <c r="C28" s="81"/>
+      <c r="D28" s="81"/>
+      <c r="E28" s="81"/>
+      <c r="F28" s="81"/>
+      <c r="G28" s="81"/>
+      <c r="H28" s="81"/>
+      <c r="I28" s="81"/>
+      <c r="J28" s="81"/>
+      <c r="K28" s="81"/>
+      <c r="L28" s="81"/>
+      <c r="M28" s="81"/>
+      <c r="N28" s="82"/>
     </row>
     <row r="29" spans="1:14" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="101"/>
-      <c r="B29" s="102"/>
-      <c r="C29" s="102"/>
-      <c r="D29" s="102"/>
-      <c r="E29" s="102"/>
-      <c r="F29" s="102"/>
-      <c r="G29" s="102"/>
-      <c r="H29" s="102"/>
-      <c r="I29" s="102"/>
-      <c r="J29" s="102"/>
-      <c r="K29" s="102"/>
-      <c r="L29" s="102"/>
-      <c r="M29" s="102"/>
-      <c r="N29" s="103"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="81"/>
+      <c r="C29" s="81"/>
+      <c r="D29" s="81"/>
+      <c r="E29" s="81"/>
+      <c r="F29" s="81"/>
+      <c r="G29" s="81"/>
+      <c r="H29" s="81"/>
+      <c r="I29" s="81"/>
+      <c r="J29" s="81"/>
+      <c r="K29" s="81"/>
+      <c r="L29" s="81"/>
+      <c r="M29" s="81"/>
+      <c r="N29" s="82"/>
     </row>
     <row r="30" spans="1:14" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="104"/>
-      <c r="B30" s="105"/>
-      <c r="C30" s="105"/>
-      <c r="D30" s="105"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="105"/>
-      <c r="G30" s="105"/>
-      <c r="H30" s="105"/>
-      <c r="I30" s="105"/>
-      <c r="J30" s="105"/>
-      <c r="K30" s="105"/>
-      <c r="L30" s="105"/>
-      <c r="M30" s="105"/>
-      <c r="N30" s="106"/>
+      <c r="A30" s="83"/>
+      <c r="B30" s="84"/>
+      <c r="C30" s="84"/>
+      <c r="D30" s="84"/>
+      <c r="E30" s="84"/>
+      <c r="F30" s="84"/>
+      <c r="G30" s="84"/>
+      <c r="H30" s="84"/>
+      <c r="I30" s="84"/>
+      <c r="J30" s="84"/>
+      <c r="K30" s="84"/>
+      <c r="L30" s="84"/>
+      <c r="M30" s="84"/>
+      <c r="N30" s="85"/>
     </row>
     <row r="31" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="95" t="s">
+      <c r="A31" s="74" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="96"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="H31" s="96"/>
-      <c r="I31" s="96"/>
-      <c r="J31" s="96"/>
-      <c r="K31" s="97"/>
-      <c r="L31" s="95" t="s">
+      <c r="B31" s="75"/>
+      <c r="C31" s="75"/>
+      <c r="D31" s="75"/>
+      <c r="E31" s="75"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="75"/>
+      <c r="J31" s="75"/>
+      <c r="K31" s="76"/>
+      <c r="L31" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="M31" s="96"/>
-      <c r="N31" s="97"/>
+      <c r="M31" s="75"/>
+      <c r="N31" s="76"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A32" s="112" t="s">
+      <c r="A32" s="53" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="113"/>
-      <c r="C32" s="114"/>
-      <c r="D32" s="118" t="s">
+      <c r="B32" s="54"/>
+      <c r="C32" s="55"/>
+      <c r="D32" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="E32" s="118"/>
-      <c r="F32" s="118"/>
-      <c r="G32" s="119" t="s">
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="H32" s="120"/>
-      <c r="I32" s="120"/>
-      <c r="J32" s="120"/>
-      <c r="K32" s="121"/>
-      <c r="L32" s="84" t="s">
+      <c r="H32" s="61"/>
+      <c r="I32" s="61"/>
+      <c r="J32" s="61"/>
+      <c r="K32" s="62"/>
+      <c r="L32" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="M32" s="86" t="s">
+      <c r="M32" s="65" t="s">
         <v>61</v>
       </c>
-      <c r="N32" s="88" t="s">
+      <c r="N32" s="67" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A33" s="115"/>
-      <c r="B33" s="116"/>
-      <c r="C33" s="117"/>
+      <c r="A33" s="56"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="58"/>
       <c r="D33" s="3" t="s">
         <v>42</v>
       </c>
@@ -2562,20 +2567,20 @@
       <c r="I33" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="J33" s="90" t="s">
+      <c r="J33" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="K33" s="91"/>
-      <c r="L33" s="85"/>
-      <c r="M33" s="87"/>
-      <c r="N33" s="89"/>
+      <c r="K33" s="70"/>
+      <c r="L33" s="64"/>
+      <c r="M33" s="66"/>
+      <c r="N33" s="68"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A34" s="107" t="s">
+      <c r="A34" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B34" s="108"/>
-      <c r="C34" s="109"/>
+      <c r="B34" s="44"/>
+      <c r="C34" s="45"/>
       <c r="D34" s="17"/>
       <c r="E34" s="18"/>
       <c r="F34" s="17"/>
@@ -2585,21 +2590,21 @@
         <f>IF(H34="","",C$14-H34)</f>
         <v/>
       </c>
-      <c r="J34" s="110" t="str">
+      <c r="J34" s="46" t="str">
         <f>IF(OR(H34="",F34=""),"",E34-H34)</f>
         <v/>
       </c>
-      <c r="K34" s="111"/>
+      <c r="K34" s="47"/>
       <c r="L34" s="23"/>
       <c r="M34" s="24"/>
       <c r="N34" s="9"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A35" s="107" t="s">
+      <c r="A35" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="B35" s="108"/>
-      <c r="C35" s="109"/>
+      <c r="B35" s="44"/>
+      <c r="C35" s="45"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
       <c r="F35" s="17"/>
@@ -2609,21 +2614,21 @@
         <f t="shared" ref="I35:I42" si="0">IF(H35="","",C$14-H35)</f>
         <v/>
       </c>
-      <c r="J35" s="110" t="str">
+      <c r="J35" s="46" t="str">
         <f t="shared" ref="J35:J42" si="1">IF(OR(H35="",F35=""),"",E35-H35)</f>
         <v/>
       </c>
-      <c r="K35" s="111"/>
+      <c r="K35" s="47"/>
       <c r="L35" s="23"/>
       <c r="M35" s="24"/>
       <c r="N35" s="9"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A36" s="107" t="s">
+      <c r="A36" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="108"/>
-      <c r="C36" s="109"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="45"/>
       <c r="D36" s="17"/>
       <c r="E36" s="18"/>
       <c r="F36" s="17"/>
@@ -2633,21 +2638,21 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J36" s="110" t="str">
+      <c r="J36" s="46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K36" s="111"/>
+      <c r="K36" s="47"/>
       <c r="L36" s="23"/>
       <c r="M36" s="22"/>
       <c r="N36" s="25"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A37" s="107" t="s">
+      <c r="A37" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="108"/>
-      <c r="C37" s="109"/>
+      <c r="B37" s="44"/>
+      <c r="C37" s="45"/>
       <c r="D37" s="17"/>
       <c r="E37" s="18"/>
       <c r="F37" s="17"/>
@@ -2657,21 +2662,21 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J37" s="110" t="str">
+      <c r="J37" s="46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K37" s="111"/>
+      <c r="K37" s="47"/>
       <c r="L37" s="10"/>
       <c r="M37" s="7"/>
       <c r="N37" s="11"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A38" s="107" t="s">
+      <c r="A38" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="108"/>
-      <c r="C38" s="109"/>
+      <c r="B38" s="44"/>
+      <c r="C38" s="45"/>
       <c r="D38" s="17"/>
       <c r="E38" s="18"/>
       <c r="F38" s="17"/>
@@ -2681,21 +2686,21 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J38" s="110" t="str">
+      <c r="J38" s="46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K38" s="111"/>
+      <c r="K38" s="47"/>
       <c r="L38" s="10"/>
       <c r="M38" s="7"/>
       <c r="N38" s="11"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A39" s="107" t="s">
+      <c r="A39" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="108"/>
-      <c r="C39" s="109"/>
+      <c r="B39" s="44"/>
+      <c r="C39" s="45"/>
       <c r="D39" s="17"/>
       <c r="E39" s="18"/>
       <c r="F39" s="17"/>
@@ -2705,21 +2710,21 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J39" s="110" t="str">
+      <c r="J39" s="46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K39" s="111"/>
+      <c r="K39" s="47"/>
       <c r="L39" s="10"/>
       <c r="M39" s="7"/>
       <c r="N39" s="11"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A40" s="107" t="s">
+      <c r="A40" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="B40" s="108"/>
-      <c r="C40" s="109"/>
+      <c r="B40" s="44"/>
+      <c r="C40" s="45"/>
       <c r="D40" s="17"/>
       <c r="E40" s="18"/>
       <c r="F40" s="17"/>
@@ -2729,21 +2734,21 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J40" s="110" t="str">
+      <c r="J40" s="46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K40" s="111"/>
+      <c r="K40" s="47"/>
       <c r="L40" s="10"/>
       <c r="M40" s="7"/>
       <c r="N40" s="11"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A41" s="107" t="s">
+      <c r="A41" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="108"/>
-      <c r="C41" s="109"/>
+      <c r="B41" s="44"/>
+      <c r="C41" s="45"/>
       <c r="D41" s="17"/>
       <c r="E41" s="18"/>
       <c r="F41" s="17"/>
@@ -2753,21 +2758,21 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J41" s="110" t="str">
+      <c r="J41" s="46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K41" s="111"/>
+      <c r="K41" s="47"/>
       <c r="L41" s="10"/>
       <c r="M41" s="7"/>
       <c r="N41" s="11"/>
     </row>
     <row r="42" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="122" t="s">
+      <c r="A42" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B42" s="123"/>
-      <c r="C42" s="124"/>
+      <c r="B42" s="49"/>
+      <c r="C42" s="50"/>
       <c r="D42" s="19"/>
       <c r="E42" s="20"/>
       <c r="F42" s="19"/>
@@ -2777,430 +2782,430 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J42" s="125" t="str">
+      <c r="J42" s="51" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K42" s="126"/>
+      <c r="K42" s="52"/>
       <c r="L42" s="12"/>
       <c r="M42" s="8"/>
       <c r="N42" s="13"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A43" s="67" t="s">
+      <c r="A43" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="B43" s="68"/>
-      <c r="C43" s="68"/>
-      <c r="D43" s="68"/>
-      <c r="E43" s="68"/>
-      <c r="F43" s="68"/>
-      <c r="G43" s="68"/>
-      <c r="H43" s="68"/>
-      <c r="I43" s="68"/>
-      <c r="J43" s="68"/>
-      <c r="K43" s="68"/>
-      <c r="L43" s="68"/>
-      <c r="M43" s="68"/>
-      <c r="N43" s="69"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="27"/>
+      <c r="L43" s="27"/>
+      <c r="M43" s="27"/>
+      <c r="N43" s="28"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A44" s="137" t="s">
+      <c r="A44" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="B44" s="65"/>
-      <c r="C44" s="65"/>
-      <c r="D44" s="65" t="s">
+      <c r="B44" s="41"/>
+      <c r="C44" s="41"/>
+      <c r="D44" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="E44" s="65"/>
-      <c r="F44" s="65"/>
-      <c r="G44" s="65" t="s">
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="H44" s="65"/>
-      <c r="I44" s="65" t="s">
+      <c r="H44" s="41"/>
+      <c r="I44" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="J44" s="65"/>
-      <c r="K44" s="65" t="s">
+      <c r="J44" s="41"/>
+      <c r="K44" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="L44" s="65"/>
-      <c r="M44" s="65" t="s">
+      <c r="L44" s="41"/>
+      <c r="M44" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="N44" s="138"/>
+      <c r="N44" s="42"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A45" s="133"/>
-      <c r="B45" s="134"/>
-      <c r="C45" s="134"/>
-      <c r="D45" s="134"/>
-      <c r="E45" s="134"/>
-      <c r="F45" s="134"/>
-      <c r="G45" s="135"/>
-      <c r="H45" s="135"/>
-      <c r="I45" s="134"/>
-      <c r="J45" s="134"/>
-      <c r="K45" s="64"/>
-      <c r="L45" s="64"/>
-      <c r="M45" s="64"/>
-      <c r="N45" s="136"/>
+      <c r="A45" s="35"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="36"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36"/>
+      <c r="F45" s="36"/>
+      <c r="G45" s="37"/>
+      <c r="H45" s="37"/>
+      <c r="I45" s="36"/>
+      <c r="J45" s="36"/>
+      <c r="K45" s="38"/>
+      <c r="L45" s="38"/>
+      <c r="M45" s="38"/>
+      <c r="N45" s="39"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A46" s="67" t="s">
+      <c r="A46" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B46" s="68"/>
-      <c r="C46" s="68"/>
-      <c r="D46" s="68"/>
-      <c r="E46" s="68"/>
-      <c r="F46" s="68"/>
-      <c r="G46" s="68"/>
-      <c r="H46" s="68"/>
-      <c r="I46" s="68"/>
-      <c r="J46" s="68"/>
-      <c r="K46" s="68"/>
-      <c r="L46" s="68"/>
-      <c r="M46" s="68"/>
-      <c r="N46" s="69"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="27"/>
+      <c r="K46" s="27"/>
+      <c r="L46" s="27"/>
+      <c r="M46" s="27"/>
+      <c r="N46" s="28"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A47" s="127"/>
-      <c r="B47" s="128"/>
-      <c r="C47" s="128"/>
-      <c r="D47" s="128"/>
-      <c r="E47" s="128"/>
-      <c r="F47" s="128"/>
-      <c r="G47" s="128"/>
-      <c r="H47" s="128"/>
-      <c r="I47" s="128"/>
-      <c r="J47" s="128"/>
-      <c r="K47" s="128"/>
-      <c r="L47" s="128"/>
-      <c r="M47" s="128"/>
-      <c r="N47" s="129"/>
+      <c r="A47" s="29"/>
+      <c r="B47" s="30"/>
+      <c r="C47" s="30"/>
+      <c r="D47" s="30"/>
+      <c r="E47" s="30"/>
+      <c r="F47" s="30"/>
+      <c r="G47" s="30"/>
+      <c r="H47" s="30"/>
+      <c r="I47" s="30"/>
+      <c r="J47" s="30"/>
+      <c r="K47" s="30"/>
+      <c r="L47" s="30"/>
+      <c r="M47" s="30"/>
+      <c r="N47" s="31"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A48" s="127"/>
-      <c r="B48" s="128"/>
-      <c r="C48" s="128"/>
-      <c r="D48" s="128"/>
-      <c r="E48" s="128"/>
-      <c r="F48" s="128"/>
-      <c r="G48" s="128"/>
-      <c r="H48" s="128"/>
-      <c r="I48" s="128"/>
-      <c r="J48" s="128"/>
-      <c r="K48" s="128"/>
-      <c r="L48" s="128"/>
-      <c r="M48" s="128"/>
-      <c r="N48" s="129"/>
+      <c r="A48" s="29"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="30"/>
+      <c r="D48" s="30"/>
+      <c r="E48" s="30"/>
+      <c r="F48" s="30"/>
+      <c r="G48" s="30"/>
+      <c r="H48" s="30"/>
+      <c r="I48" s="30"/>
+      <c r="J48" s="30"/>
+      <c r="K48" s="30"/>
+      <c r="L48" s="30"/>
+      <c r="M48" s="30"/>
+      <c r="N48" s="31"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A49" s="127"/>
-      <c r="B49" s="128"/>
-      <c r="C49" s="128"/>
-      <c r="D49" s="128"/>
-      <c r="E49" s="128"/>
-      <c r="F49" s="128"/>
-      <c r="G49" s="128"/>
-      <c r="H49" s="128"/>
-      <c r="I49" s="128"/>
-      <c r="J49" s="128"/>
-      <c r="K49" s="128"/>
-      <c r="L49" s="128"/>
-      <c r="M49" s="128"/>
-      <c r="N49" s="129"/>
+      <c r="A49" s="29"/>
+      <c r="B49" s="30"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="30"/>
+      <c r="E49" s="30"/>
+      <c r="F49" s="30"/>
+      <c r="G49" s="30"/>
+      <c r="H49" s="30"/>
+      <c r="I49" s="30"/>
+      <c r="J49" s="30"/>
+      <c r="K49" s="30"/>
+      <c r="L49" s="30"/>
+      <c r="M49" s="30"/>
+      <c r="N49" s="31"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A50" s="127"/>
-      <c r="B50" s="128"/>
-      <c r="C50" s="128"/>
-      <c r="D50" s="128"/>
-      <c r="E50" s="128"/>
-      <c r="F50" s="128"/>
-      <c r="G50" s="128"/>
-      <c r="H50" s="128"/>
-      <c r="I50" s="128"/>
-      <c r="J50" s="128"/>
-      <c r="K50" s="128"/>
-      <c r="L50" s="128"/>
-      <c r="M50" s="128"/>
-      <c r="N50" s="129"/>
+      <c r="A50" s="29"/>
+      <c r="B50" s="30"/>
+      <c r="C50" s="30"/>
+      <c r="D50" s="30"/>
+      <c r="E50" s="30"/>
+      <c r="F50" s="30"/>
+      <c r="G50" s="30"/>
+      <c r="H50" s="30"/>
+      <c r="I50" s="30"/>
+      <c r="J50" s="30"/>
+      <c r="K50" s="30"/>
+      <c r="L50" s="30"/>
+      <c r="M50" s="30"/>
+      <c r="N50" s="31"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A51" s="127"/>
-      <c r="B51" s="128"/>
-      <c r="C51" s="128"/>
-      <c r="D51" s="128"/>
-      <c r="E51" s="128"/>
-      <c r="F51" s="128"/>
-      <c r="G51" s="128"/>
-      <c r="H51" s="128"/>
-      <c r="I51" s="128"/>
-      <c r="J51" s="128"/>
-      <c r="K51" s="128"/>
-      <c r="L51" s="128"/>
-      <c r="M51" s="128"/>
-      <c r="N51" s="129"/>
+      <c r="A51" s="29"/>
+      <c r="B51" s="30"/>
+      <c r="C51" s="30"/>
+      <c r="D51" s="30"/>
+      <c r="E51" s="30"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
+      <c r="I51" s="30"/>
+      <c r="J51" s="30"/>
+      <c r="K51" s="30"/>
+      <c r="L51" s="30"/>
+      <c r="M51" s="30"/>
+      <c r="N51" s="31"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A52" s="127"/>
-      <c r="B52" s="128"/>
-      <c r="C52" s="128"/>
-      <c r="D52" s="128"/>
-      <c r="E52" s="128"/>
-      <c r="F52" s="128"/>
-      <c r="G52" s="128"/>
-      <c r="H52" s="128"/>
-      <c r="I52" s="128"/>
-      <c r="J52" s="128"/>
-      <c r="K52" s="128"/>
-      <c r="L52" s="128"/>
-      <c r="M52" s="128"/>
-      <c r="N52" s="129"/>
+      <c r="A52" s="29"/>
+      <c r="B52" s="30"/>
+      <c r="C52" s="30"/>
+      <c r="D52" s="30"/>
+      <c r="E52" s="30"/>
+      <c r="F52" s="30"/>
+      <c r="G52" s="30"/>
+      <c r="H52" s="30"/>
+      <c r="I52" s="30"/>
+      <c r="J52" s="30"/>
+      <c r="K52" s="30"/>
+      <c r="L52" s="30"/>
+      <c r="M52" s="30"/>
+      <c r="N52" s="31"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A53" s="127"/>
-      <c r="B53" s="128"/>
-      <c r="C53" s="128"/>
-      <c r="D53" s="128"/>
-      <c r="E53" s="128"/>
-      <c r="F53" s="128"/>
-      <c r="G53" s="128"/>
-      <c r="H53" s="128"/>
-      <c r="I53" s="128"/>
-      <c r="J53" s="128"/>
-      <c r="K53" s="128"/>
-      <c r="L53" s="128"/>
-      <c r="M53" s="128"/>
-      <c r="N53" s="129"/>
+      <c r="A53" s="29"/>
+      <c r="B53" s="30"/>
+      <c r="C53" s="30"/>
+      <c r="D53" s="30"/>
+      <c r="E53" s="30"/>
+      <c r="F53" s="30"/>
+      <c r="G53" s="30"/>
+      <c r="H53" s="30"/>
+      <c r="I53" s="30"/>
+      <c r="J53" s="30"/>
+      <c r="K53" s="30"/>
+      <c r="L53" s="30"/>
+      <c r="M53" s="30"/>
+      <c r="N53" s="31"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A54" s="127"/>
-      <c r="B54" s="128"/>
-      <c r="C54" s="128"/>
-      <c r="D54" s="128"/>
-      <c r="E54" s="128"/>
-      <c r="F54" s="128"/>
-      <c r="G54" s="128"/>
-      <c r="H54" s="128"/>
-      <c r="I54" s="128"/>
-      <c r="J54" s="128"/>
-      <c r="K54" s="128"/>
-      <c r="L54" s="128"/>
-      <c r="M54" s="128"/>
-      <c r="N54" s="129"/>
+      <c r="A54" s="29"/>
+      <c r="B54" s="30"/>
+      <c r="C54" s="30"/>
+      <c r="D54" s="30"/>
+      <c r="E54" s="30"/>
+      <c r="F54" s="30"/>
+      <c r="G54" s="30"/>
+      <c r="H54" s="30"/>
+      <c r="I54" s="30"/>
+      <c r="J54" s="30"/>
+      <c r="K54" s="30"/>
+      <c r="L54" s="30"/>
+      <c r="M54" s="30"/>
+      <c r="N54" s="31"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A55" s="127"/>
-      <c r="B55" s="128"/>
-      <c r="C55" s="128"/>
-      <c r="D55" s="128"/>
-      <c r="E55" s="128"/>
-      <c r="F55" s="128"/>
-      <c r="G55" s="128"/>
-      <c r="H55" s="128"/>
-      <c r="I55" s="128"/>
-      <c r="J55" s="128"/>
-      <c r="K55" s="128"/>
-      <c r="L55" s="128"/>
-      <c r="M55" s="128"/>
-      <c r="N55" s="129"/>
+      <c r="A55" s="29"/>
+      <c r="B55" s="30"/>
+      <c r="C55" s="30"/>
+      <c r="D55" s="30"/>
+      <c r="E55" s="30"/>
+      <c r="F55" s="30"/>
+      <c r="G55" s="30"/>
+      <c r="H55" s="30"/>
+      <c r="I55" s="30"/>
+      <c r="J55" s="30"/>
+      <c r="K55" s="30"/>
+      <c r="L55" s="30"/>
+      <c r="M55" s="30"/>
+      <c r="N55" s="31"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A56" s="127"/>
-      <c r="B56" s="128"/>
-      <c r="C56" s="128"/>
-      <c r="D56" s="128"/>
-      <c r="E56" s="128"/>
-      <c r="F56" s="128"/>
-      <c r="G56" s="128"/>
-      <c r="H56" s="128"/>
-      <c r="I56" s="128"/>
-      <c r="J56" s="128"/>
-      <c r="K56" s="128"/>
-      <c r="L56" s="128"/>
-      <c r="M56" s="128"/>
-      <c r="N56" s="129"/>
+      <c r="A56" s="29"/>
+      <c r="B56" s="30"/>
+      <c r="C56" s="30"/>
+      <c r="D56" s="30"/>
+      <c r="E56" s="30"/>
+      <c r="F56" s="30"/>
+      <c r="G56" s="30"/>
+      <c r="H56" s="30"/>
+      <c r="I56" s="30"/>
+      <c r="J56" s="30"/>
+      <c r="K56" s="30"/>
+      <c r="L56" s="30"/>
+      <c r="M56" s="30"/>
+      <c r="N56" s="31"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A57" s="127"/>
-      <c r="B57" s="128"/>
-      <c r="C57" s="128"/>
-      <c r="D57" s="128"/>
-      <c r="E57" s="128"/>
-      <c r="F57" s="128"/>
-      <c r="G57" s="128"/>
-      <c r="H57" s="128"/>
-      <c r="I57" s="128"/>
-      <c r="J57" s="128"/>
-      <c r="K57" s="128"/>
-      <c r="L57" s="128"/>
-      <c r="M57" s="128"/>
-      <c r="N57" s="129"/>
+      <c r="A57" s="29"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="30"/>
+      <c r="D57" s="30"/>
+      <c r="E57" s="30"/>
+      <c r="F57" s="30"/>
+      <c r="G57" s="30"/>
+      <c r="H57" s="30"/>
+      <c r="I57" s="30"/>
+      <c r="J57" s="30"/>
+      <c r="K57" s="30"/>
+      <c r="L57" s="30"/>
+      <c r="M57" s="30"/>
+      <c r="N57" s="31"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A58" s="127"/>
-      <c r="B58" s="128"/>
-      <c r="C58" s="128"/>
-      <c r="D58" s="128"/>
-      <c r="E58" s="128"/>
-      <c r="F58" s="128"/>
-      <c r="G58" s="128"/>
-      <c r="H58" s="128"/>
-      <c r="I58" s="128"/>
-      <c r="J58" s="128"/>
-      <c r="K58" s="128"/>
-      <c r="L58" s="128"/>
-      <c r="M58" s="128"/>
-      <c r="N58" s="129"/>
+      <c r="A58" s="29"/>
+      <c r="B58" s="30"/>
+      <c r="C58" s="30"/>
+      <c r="D58" s="30"/>
+      <c r="E58" s="30"/>
+      <c r="F58" s="30"/>
+      <c r="G58" s="30"/>
+      <c r="H58" s="30"/>
+      <c r="I58" s="30"/>
+      <c r="J58" s="30"/>
+      <c r="K58" s="30"/>
+      <c r="L58" s="30"/>
+      <c r="M58" s="30"/>
+      <c r="N58" s="31"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A59" s="127"/>
-      <c r="B59" s="128"/>
-      <c r="C59" s="128"/>
-      <c r="D59" s="128"/>
-      <c r="E59" s="128"/>
-      <c r="F59" s="128"/>
-      <c r="G59" s="128"/>
-      <c r="H59" s="128"/>
-      <c r="I59" s="128"/>
-      <c r="J59" s="128"/>
-      <c r="K59" s="128"/>
-      <c r="L59" s="128"/>
-      <c r="M59" s="128"/>
-      <c r="N59" s="129"/>
+      <c r="A59" s="29"/>
+      <c r="B59" s="30"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="30"/>
+      <c r="E59" s="30"/>
+      <c r="F59" s="30"/>
+      <c r="G59" s="30"/>
+      <c r="H59" s="30"/>
+      <c r="I59" s="30"/>
+      <c r="J59" s="30"/>
+      <c r="K59" s="30"/>
+      <c r="L59" s="30"/>
+      <c r="M59" s="30"/>
+      <c r="N59" s="31"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A60" s="127"/>
-      <c r="B60" s="128"/>
-      <c r="C60" s="128"/>
-      <c r="D60" s="128"/>
-      <c r="E60" s="128"/>
-      <c r="F60" s="128"/>
-      <c r="G60" s="128"/>
-      <c r="H60" s="128"/>
-      <c r="I60" s="128"/>
-      <c r="J60" s="128"/>
-      <c r="K60" s="128"/>
-      <c r="L60" s="128"/>
-      <c r="M60" s="128"/>
-      <c r="N60" s="129"/>
+      <c r="A60" s="29"/>
+      <c r="B60" s="30"/>
+      <c r="C60" s="30"/>
+      <c r="D60" s="30"/>
+      <c r="E60" s="30"/>
+      <c r="F60" s="30"/>
+      <c r="G60" s="30"/>
+      <c r="H60" s="30"/>
+      <c r="I60" s="30"/>
+      <c r="J60" s="30"/>
+      <c r="K60" s="30"/>
+      <c r="L60" s="30"/>
+      <c r="M60" s="30"/>
+      <c r="N60" s="31"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A61" s="127"/>
-      <c r="B61" s="128"/>
-      <c r="C61" s="128"/>
-      <c r="D61" s="128"/>
-      <c r="E61" s="128"/>
-      <c r="F61" s="128"/>
-      <c r="G61" s="128"/>
-      <c r="H61" s="128"/>
-      <c r="I61" s="128"/>
-      <c r="J61" s="128"/>
-      <c r="K61" s="128"/>
-      <c r="L61" s="128"/>
-      <c r="M61" s="128"/>
-      <c r="N61" s="129"/>
+      <c r="A61" s="29"/>
+      <c r="B61" s="30"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="30"/>
+      <c r="E61" s="30"/>
+      <c r="F61" s="30"/>
+      <c r="G61" s="30"/>
+      <c r="H61" s="30"/>
+      <c r="I61" s="30"/>
+      <c r="J61" s="30"/>
+      <c r="K61" s="30"/>
+      <c r="L61" s="30"/>
+      <c r="M61" s="30"/>
+      <c r="N61" s="31"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A62" s="127"/>
-      <c r="B62" s="128"/>
-      <c r="C62" s="128"/>
-      <c r="D62" s="128"/>
-      <c r="E62" s="128"/>
-      <c r="F62" s="128"/>
-      <c r="G62" s="128"/>
-      <c r="H62" s="128"/>
-      <c r="I62" s="128"/>
-      <c r="J62" s="128"/>
-      <c r="K62" s="128"/>
-      <c r="L62" s="128"/>
-      <c r="M62" s="128"/>
-      <c r="N62" s="129"/>
+      <c r="A62" s="29"/>
+      <c r="B62" s="30"/>
+      <c r="C62" s="30"/>
+      <c r="D62" s="30"/>
+      <c r="E62" s="30"/>
+      <c r="F62" s="30"/>
+      <c r="G62" s="30"/>
+      <c r="H62" s="30"/>
+      <c r="I62" s="30"/>
+      <c r="J62" s="30"/>
+      <c r="K62" s="30"/>
+      <c r="L62" s="30"/>
+      <c r="M62" s="30"/>
+      <c r="N62" s="31"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A63" s="127"/>
-      <c r="B63" s="128"/>
-      <c r="C63" s="128"/>
-      <c r="D63" s="128"/>
-      <c r="E63" s="128"/>
-      <c r="F63" s="128"/>
-      <c r="G63" s="128"/>
-      <c r="H63" s="128"/>
-      <c r="I63" s="128"/>
-      <c r="J63" s="128"/>
-      <c r="K63" s="128"/>
-      <c r="L63" s="128"/>
-      <c r="M63" s="128"/>
-      <c r="N63" s="129"/>
+      <c r="A63" s="29"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="30"/>
+      <c r="D63" s="30"/>
+      <c r="E63" s="30"/>
+      <c r="F63" s="30"/>
+      <c r="G63" s="30"/>
+      <c r="H63" s="30"/>
+      <c r="I63" s="30"/>
+      <c r="J63" s="30"/>
+      <c r="K63" s="30"/>
+      <c r="L63" s="30"/>
+      <c r="M63" s="30"/>
+      <c r="N63" s="31"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A64" s="127"/>
-      <c r="B64" s="128"/>
-      <c r="C64" s="128"/>
-      <c r="D64" s="128"/>
-      <c r="E64" s="128"/>
-      <c r="F64" s="128"/>
-      <c r="G64" s="128"/>
-      <c r="H64" s="128"/>
-      <c r="I64" s="128"/>
-      <c r="J64" s="128"/>
-      <c r="K64" s="128"/>
-      <c r="L64" s="128"/>
-      <c r="M64" s="128"/>
-      <c r="N64" s="129"/>
+      <c r="A64" s="29"/>
+      <c r="B64" s="30"/>
+      <c r="C64" s="30"/>
+      <c r="D64" s="30"/>
+      <c r="E64" s="30"/>
+      <c r="F64" s="30"/>
+      <c r="G64" s="30"/>
+      <c r="H64" s="30"/>
+      <c r="I64" s="30"/>
+      <c r="J64" s="30"/>
+      <c r="K64" s="30"/>
+      <c r="L64" s="30"/>
+      <c r="M64" s="30"/>
+      <c r="N64" s="31"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A65" s="127"/>
-      <c r="B65" s="128"/>
-      <c r="C65" s="128"/>
-      <c r="D65" s="128"/>
-      <c r="E65" s="128"/>
-      <c r="F65" s="128"/>
-      <c r="G65" s="128"/>
-      <c r="H65" s="128"/>
-      <c r="I65" s="128"/>
-      <c r="J65" s="128"/>
-      <c r="K65" s="128"/>
-      <c r="L65" s="128"/>
-      <c r="M65" s="128"/>
-      <c r="N65" s="129"/>
+      <c r="A65" s="29"/>
+      <c r="B65" s="30"/>
+      <c r="C65" s="30"/>
+      <c r="D65" s="30"/>
+      <c r="E65" s="30"/>
+      <c r="F65" s="30"/>
+      <c r="G65" s="30"/>
+      <c r="H65" s="30"/>
+      <c r="I65" s="30"/>
+      <c r="J65" s="30"/>
+      <c r="K65" s="30"/>
+      <c r="L65" s="30"/>
+      <c r="M65" s="30"/>
+      <c r="N65" s="31"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A66" s="127"/>
-      <c r="B66" s="128"/>
-      <c r="C66" s="128"/>
-      <c r="D66" s="128"/>
-      <c r="E66" s="128"/>
-      <c r="F66" s="128"/>
-      <c r="G66" s="128"/>
-      <c r="H66" s="128"/>
-      <c r="I66" s="128"/>
-      <c r="J66" s="128"/>
-      <c r="K66" s="128"/>
-      <c r="L66" s="128"/>
-      <c r="M66" s="128"/>
-      <c r="N66" s="129"/>
+      <c r="A66" s="29"/>
+      <c r="B66" s="30"/>
+      <c r="C66" s="30"/>
+      <c r="D66" s="30"/>
+      <c r="E66" s="30"/>
+      <c r="F66" s="30"/>
+      <c r="G66" s="30"/>
+      <c r="H66" s="30"/>
+      <c r="I66" s="30"/>
+      <c r="J66" s="30"/>
+      <c r="K66" s="30"/>
+      <c r="L66" s="30"/>
+      <c r="M66" s="30"/>
+      <c r="N66" s="31"/>
     </row>
     <row r="67" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="130"/>
-      <c r="B67" s="131"/>
-      <c r="C67" s="131"/>
-      <c r="D67" s="131"/>
-      <c r="E67" s="131"/>
-      <c r="F67" s="131"/>
-      <c r="G67" s="131"/>
-      <c r="H67" s="131"/>
-      <c r="I67" s="131"/>
-      <c r="J67" s="131"/>
-      <c r="K67" s="131"/>
-      <c r="L67" s="131"/>
-      <c r="M67" s="131"/>
-      <c r="N67" s="132"/>
+      <c r="A67" s="32"/>
+      <c r="B67" s="33"/>
+      <c r="C67" s="33"/>
+      <c r="D67" s="33"/>
+      <c r="E67" s="33"/>
+      <c r="F67" s="33"/>
+      <c r="G67" s="33"/>
+      <c r="H67" s="33"/>
+      <c r="I67" s="33"/>
+      <c r="J67" s="33"/>
+      <c r="K67" s="33"/>
+      <c r="L67" s="33"/>
+      <c r="M67" s="33"/>
+      <c r="N67" s="34"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" s="1"/>
@@ -3221,92 +3226,6 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="107">
-    <mergeCell ref="A46:N46"/>
-    <mergeCell ref="A47:N67"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="K45:L45"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="A43:N43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="A32:C33"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="L32:L33"/>
-    <mergeCell ref="M32:M33"/>
-    <mergeCell ref="N32:N33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="A18:N18"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="A20:N24"/>
-    <mergeCell ref="A25:N25"/>
-    <mergeCell ref="A26:N30"/>
-    <mergeCell ref="A31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="A10:N10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:E9"/>
-    <mergeCell ref="F8:G9"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="L9:N9"/>
     <mergeCell ref="A1:C3"/>
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:N1"/>
@@ -3328,6 +3247,92 @@
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="I5:K5"/>
     <mergeCell ref="L5:N5"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:E9"/>
+    <mergeCell ref="F8:G9"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A17:N17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="L32:L33"/>
+    <mergeCell ref="M32:M33"/>
+    <mergeCell ref="N32:N33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="A18:N18"/>
+    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="A20:N24"/>
+    <mergeCell ref="A25:N25"/>
+    <mergeCell ref="A26:N30"/>
+    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="A32:C33"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="A46:N46"/>
+    <mergeCell ref="A47:N67"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="A43:N43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:N44"/>
   </mergeCells>
   <conditionalFormatting sqref="C6">
     <cfRule type="notContainsBlanks" dxfId="7" priority="6">
@@ -3650,6 +3655,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="0a16e579-8e52-462c-b9fb-90fad13862ef">
@@ -3658,15 +3672,6 @@
     <TaxCatchAll xmlns="90a9caed-1441-4e6e-970c-7f1ae8660165" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3690,6 +3695,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{621519AB-4E14-47F6-8EE1-734F9264F5A4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{282588ED-C501-480E-90CA-BF6563DD6F5F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3698,12 +3711,4 @@
     <ds:schemaRef ds:uri="90a9caed-1441-4e6e-970c-7f1ae8660165"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{621519AB-4E14-47F6-8EE1-734F9264F5A4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>